<commit_message>
Diverse Verbesserungen bzgl. IAmbe3000RController
</commit_message>
<xml_diff>
--- a/Projektstruktur.xlsx
+++ b/Projektstruktur.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hgbir\VisualStudio_Source\repos\CsDigimodes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B13E9F8-5725-4D68-93D0-863742000711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A59355-CFD7-4FF0-8E2F-F7C8D7BA2D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="735" yWindow="735" windowWidth="26910" windowHeight="13335" xr2:uid="{1A4329D0-C53F-437D-9914-D6316396BCBD}"/>
   </bookViews>
@@ -161,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -174,6 +174,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -528,7 +531,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
@@ -549,6 +552,7 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="7"/>
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -977,6 +981,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>